<commit_message>
Reclasificar KIT DE TRANSFERENCIA V2 como Sin tiempo (ya no queda ningun curso Nuevo - revisar)
</commit_message>
<xml_diff>
--- a/Tiempo de Duracion de Cursos.xlsx
+++ b/Tiempo de Duracion de Cursos.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,12 +44,8 @@
       <i val="1"/>
       <color rgb="FF6B7280"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF2F6BE4"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -72,12 +68,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF0F0EE"/>
         <bgColor rgb="FFF0F0EE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F0FE"/>
-        <bgColor rgb="FFE8F0FE"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -132,13 +122,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -551,7 +534,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Talma Servicios Aeroportuarios · 262 cursos con "2026" · 210 con duración · 49 sin tiempo · 2 sin examen · 1 nuevos por revisar · actualizado contra reporteglobal.xlsx del día</t>
+          <t xml:space="preserve">  Talma Servicios Aeroportuarios · 262 cursos con "2026" · 210 con duración · 50 sin tiempo · 2 sin examen · 0 nuevos por revisar · actualizado contra reporteglobal.xlsx del día</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -699,7 +682,7 @@
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
     <row r="11">
@@ -791,7 +774,7 @@
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15">
@@ -860,7 +843,7 @@
         </is>
       </c>
       <c r="E17" s="8" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18">
@@ -977,7 +960,7 @@
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>1791</v>
+        <v>1813</v>
       </c>
     </row>
     <row r="23">
@@ -1236,7 +1219,7 @@
         </is>
       </c>
       <c r="E33" s="8" t="n">
-        <v>500</v>
+        <v>524</v>
       </c>
     </row>
     <row r="34">
@@ -1282,7 +1265,7 @@
         </is>
       </c>
       <c r="E35" s="8" t="n">
-        <v>2909</v>
+        <v>2932</v>
       </c>
     </row>
     <row r="36">
@@ -1305,7 +1288,7 @@
         </is>
       </c>
       <c r="E36" s="8" t="n">
-        <v>3123</v>
+        <v>3124</v>
       </c>
     </row>
     <row r="37">
@@ -1351,7 +1334,7 @@
         </is>
       </c>
       <c r="E38" s="8" t="n">
-        <v>722</v>
+        <v>725</v>
       </c>
     </row>
     <row r="39">
@@ -1608,7 +1591,7 @@
         </is>
       </c>
       <c r="E49" s="8" t="n">
-        <v>2906</v>
+        <v>2929</v>
       </c>
     </row>
     <row r="50">
@@ -1631,7 +1614,7 @@
         </is>
       </c>
       <c r="E50" s="8" t="n">
-        <v>2983</v>
+        <v>2984</v>
       </c>
     </row>
     <row r="51">
@@ -1704,7 +1687,7 @@
         </is>
       </c>
       <c r="E53" s="8" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="54">
@@ -1773,7 +1756,7 @@
         </is>
       </c>
       <c r="E56" s="8" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="57">
@@ -1796,7 +1779,7 @@
         </is>
       </c>
       <c r="E57" s="8" t="n">
-        <v>945</v>
+        <v>967</v>
       </c>
     </row>
     <row r="58">
@@ -2028,7 +2011,7 @@
         </is>
       </c>
       <c r="E67" s="8" t="n">
-        <v>1173</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="68">
@@ -2051,7 +2034,7 @@
         </is>
       </c>
       <c r="E68" s="8" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="69">
@@ -2074,7 +2057,7 @@
         </is>
       </c>
       <c r="E69" s="8" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="70">
@@ -2324,7 +2307,7 @@
         </is>
       </c>
       <c r="E79" s="11" t="n">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="80">
@@ -2399,7 +2382,7 @@
         </is>
       </c>
       <c r="E82" s="11" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="83">
@@ -2745,7 +2728,7 @@
         </is>
       </c>
       <c r="E96" s="8" t="n">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="97">
@@ -2837,7 +2820,7 @@
         </is>
       </c>
       <c r="E100" s="8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="101">
@@ -2952,7 +2935,7 @@
         </is>
       </c>
       <c r="E105" s="8" t="n">
-        <v>382</v>
+        <v>386</v>
       </c>
     </row>
     <row r="106">
@@ -3476,7 +3459,7 @@
         </is>
       </c>
       <c r="E127" s="8" t="n">
-        <v>1353</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="128">
@@ -3522,7 +3505,7 @@
         </is>
       </c>
       <c r="E129" s="8" t="n">
-        <v>1884</v>
+        <v>1906</v>
       </c>
     </row>
     <row r="130">
@@ -3545,7 +3528,7 @@
         </is>
       </c>
       <c r="E130" s="8" t="n">
-        <v>1747</v>
+        <v>1775</v>
       </c>
     </row>
     <row r="131">
@@ -3591,7 +3574,7 @@
         </is>
       </c>
       <c r="E132" s="8" t="n">
-        <v>2594</v>
+        <v>2618</v>
       </c>
     </row>
     <row r="133">
@@ -3637,7 +3620,7 @@
         </is>
       </c>
       <c r="E134" s="8" t="n">
-        <v>1867</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="135">
@@ -3660,7 +3643,7 @@
         </is>
       </c>
       <c r="E135" s="8" t="n">
-        <v>2242</v>
+        <v>2268</v>
       </c>
     </row>
     <row r="136">
@@ -3708,7 +3691,7 @@
         </is>
       </c>
       <c r="E137" s="11" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="138">
@@ -3733,32 +3716,32 @@
         </is>
       </c>
       <c r="E138" s="11" t="n">
-        <v>1660</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="12" t="inlineStr">
+      <c r="A139" s="9" t="inlineStr">
         <is>
           <t>KIT DE TRANSFERENCIA - TALMA - INICIAL _ 2026V2</t>
         </is>
       </c>
-      <c r="B139" s="12" t="inlineStr">
+      <c r="B139" s="9" t="inlineStr">
         <is>
           <t>LASA, LASA SOCIEDAD DE APOYO AEROPORTUARIO, TALMA, TALMA - ANTES LASA S.A.</t>
         </is>
       </c>
-      <c r="C139" s="13" t="inlineStr">
-        <is>
-          <t>NUEVO - REVISAR</t>
-        </is>
-      </c>
-      <c r="D139" s="13" t="inlineStr">
-        <is>
-          <t>NUEVO - REVISAR</t>
-        </is>
-      </c>
-      <c r="E139" s="14" t="n">
-        <v>94</v>
+      <c r="C139" s="10" t="inlineStr">
+        <is>
+          <t>Sin tiempo</t>
+        </is>
+      </c>
+      <c r="D139" s="10" t="inlineStr">
+        <is>
+          <t>Sin tiempo</t>
+        </is>
+      </c>
+      <c r="E139" s="11" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="140">
@@ -3988,7 +3971,7 @@
         </is>
       </c>
       <c r="E149" s="8" t="n">
-        <v>1104</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="150">
@@ -4057,7 +4040,7 @@
         </is>
       </c>
       <c r="E152" s="8" t="n">
-        <v>1085</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="153">
@@ -4080,7 +4063,7 @@
         </is>
       </c>
       <c r="E153" s="8" t="n">
-        <v>225</v>
+        <v>220</v>
       </c>
     </row>
     <row r="154">
@@ -4241,7 +4224,7 @@
         </is>
       </c>
       <c r="E160" s="8" t="n">
-        <v>2792</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="161">
@@ -4264,7 +4247,7 @@
         </is>
       </c>
       <c r="E161" s="8" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="162">
@@ -4310,7 +4293,7 @@
         </is>
       </c>
       <c r="E163" s="8" t="n">
-        <v>1119</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="164">
@@ -4471,7 +4454,7 @@
         </is>
       </c>
       <c r="E170" s="8" t="n">
-        <v>1090</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="171">
@@ -4540,7 +4523,7 @@
         </is>
       </c>
       <c r="E173" s="8" t="n">
-        <v>1229</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="174">
@@ -4586,7 +4569,7 @@
         </is>
       </c>
       <c r="E175" s="8" t="n">
-        <v>1215</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="176">
@@ -4910,7 +4893,7 @@
         </is>
       </c>
       <c r="E189" s="8" t="n">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="190">
@@ -4956,7 +4939,7 @@
         </is>
       </c>
       <c r="E191" s="8" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="192">
@@ -5025,7 +5008,7 @@
         </is>
       </c>
       <c r="E194" s="8" t="n">
-        <v>593</v>
+        <v>594</v>
       </c>
     </row>
     <row r="195">
@@ -5071,7 +5054,7 @@
         </is>
       </c>
       <c r="E196" s="8" t="n">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="197">
@@ -5117,7 +5100,7 @@
         </is>
       </c>
       <c r="E198" s="8" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="199">
@@ -5163,7 +5146,7 @@
         </is>
       </c>
       <c r="E200" s="8" t="n">
-        <v>1140</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="201">
@@ -5560,7 +5543,7 @@
         </is>
       </c>
       <c r="E217" s="8" t="n">
-        <v>1373</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="218">
@@ -5606,7 +5589,7 @@
         </is>
       </c>
       <c r="E219" s="8" t="n">
-        <v>2859</v>
+        <v>2882</v>
       </c>
     </row>
     <row r="220">
@@ -5629,7 +5612,7 @@
         </is>
       </c>
       <c r="E220" s="8" t="n">
-        <v>2787</v>
+        <v>2788</v>
       </c>
     </row>
     <row r="221">
@@ -5652,7 +5635,7 @@
         </is>
       </c>
       <c r="E221" s="8" t="n">
-        <v>2907</v>
+        <v>2929</v>
       </c>
     </row>
     <row r="222">
@@ -5698,7 +5681,7 @@
         </is>
       </c>
       <c r="E223" s="8" t="n">
-        <v>457</v>
+        <v>459</v>
       </c>
     </row>
     <row r="224">
@@ -5744,7 +5727,7 @@
         </is>
       </c>
       <c r="E225" s="8" t="n">
-        <v>2742</v>
+        <v>2766</v>
       </c>
     </row>
     <row r="226">
@@ -5813,7 +5796,7 @@
         </is>
       </c>
       <c r="E228" s="8" t="n">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="229">
@@ -5859,7 +5842,7 @@
         </is>
       </c>
       <c r="E230" s="8" t="n">
-        <v>3013</v>
+        <v>3036</v>
       </c>
     </row>
     <row r="231">
@@ -5905,7 +5888,7 @@
         </is>
       </c>
       <c r="E232" s="8" t="n">
-        <v>2727</v>
+        <v>2728</v>
       </c>
     </row>
     <row r="233">
@@ -5928,7 +5911,7 @@
         </is>
       </c>
       <c r="E233" s="8" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="234">
@@ -5974,7 +5957,7 @@
         </is>
       </c>
       <c r="E235" s="8" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="236">
@@ -6043,7 +6026,7 @@
         </is>
       </c>
       <c r="E238" s="8" t="n">
-        <v>526</v>
+        <v>549</v>
       </c>
     </row>
     <row r="239">
@@ -6066,7 +6049,7 @@
         </is>
       </c>
       <c r="E239" s="8" t="n">
-        <v>1223</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="240">
@@ -6089,7 +6072,7 @@
         </is>
       </c>
       <c r="E240" s="8" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="241">
@@ -6250,7 +6233,7 @@
         </is>
       </c>
       <c r="E247" s="8" t="n">
-        <v>1130</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="248">
@@ -6344,7 +6327,7 @@
         </is>
       </c>
       <c r="E251" s="8" t="n">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="252">
@@ -6505,7 +6488,7 @@
         </is>
       </c>
       <c r="E258" s="8" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="259">
@@ -6528,7 +6511,7 @@
         </is>
       </c>
       <c r="E259" s="8" t="n">
-        <v>222</v>
+        <v>226</v>
       </c>
     </row>
     <row r="260">
@@ -6599,7 +6582,7 @@
         </is>
       </c>
       <c r="E262" s="11" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="263">
@@ -6691,7 +6674,7 @@
         </is>
       </c>
       <c r="E266" s="8" t="n">
-        <v>1245</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="267">

</xml_diff>

<commit_message>
Actualizar registros 2026 contra reporteador del dia (sin cambios de duracion ni cursos nuevos)
</commit_message>
<xml_diff>
--- a/Tiempo de Duracion de Cursos.xlsx
+++ b/Tiempo de Duracion de Cursos.xlsx
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>1232</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="7">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="E7" s="8" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8">
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="9">
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="E9" s="8" t="n">
-        <v>71</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10">
@@ -682,7 +682,7 @@
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>325</v>
+        <v>332</v>
       </c>
     </row>
     <row r="11">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="E13" s="8" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="E15" s="8" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16">
@@ -820,7 +820,7 @@
         </is>
       </c>
       <c r="E16" s="8" t="n">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="17">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="E17" s="8" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18">
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="E19" s="8" t="n">
-        <v>291</v>
+        <v>295</v>
       </c>
     </row>
     <row r="20">
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>1813</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="23">
@@ -1006,7 +1006,7 @@
         </is>
       </c>
       <c r="E24" s="8" t="n">
-        <v>1430</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="25">
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="E27" s="8" t="n">
-        <v>1911</v>
+        <v>1972</v>
       </c>
     </row>
     <row r="28">
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="E28" s="11" t="n">
-        <v>477</v>
+        <v>489</v>
       </c>
     </row>
     <row r="29">
@@ -1148,7 +1148,7 @@
         </is>
       </c>
       <c r="E30" s="11" t="n">
-        <v>511</v>
+        <v>523</v>
       </c>
     </row>
     <row r="31">
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="E31" s="8" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="32">
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="E32" s="11" t="n">
-        <v>1463</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="33">
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="E33" s="8" t="n">
-        <v>524</v>
+        <v>552</v>
       </c>
     </row>
     <row r="34">
@@ -1265,7 +1265,7 @@
         </is>
       </c>
       <c r="E35" s="8" t="n">
-        <v>2932</v>
+        <v>3020</v>
       </c>
     </row>
     <row r="36">
@@ -1288,7 +1288,7 @@
         </is>
       </c>
       <c r="E36" s="8" t="n">
-        <v>3124</v>
+        <v>3128</v>
       </c>
     </row>
     <row r="37">
@@ -1334,7 +1334,7 @@
         </is>
       </c>
       <c r="E38" s="8" t="n">
-        <v>725</v>
+        <v>774</v>
       </c>
     </row>
     <row r="39">
@@ -1380,7 +1380,7 @@
         </is>
       </c>
       <c r="E40" s="8" t="n">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="41">
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="E41" s="8" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="42">
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="E45" s="8" t="n">
-        <v>502</v>
+        <v>514</v>
       </c>
     </row>
     <row r="46">
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="E47" s="11" t="n">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="48">
@@ -1591,7 +1591,7 @@
         </is>
       </c>
       <c r="E49" s="8" t="n">
-        <v>2929</v>
+        <v>3017</v>
       </c>
     </row>
     <row r="50">
@@ -1614,7 +1614,7 @@
         </is>
       </c>
       <c r="E50" s="8" t="n">
-        <v>2984</v>
+        <v>2988</v>
       </c>
     </row>
     <row r="51">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="E51" s="11" t="n">
-        <v>386</v>
+        <v>394</v>
       </c>
     </row>
     <row r="52">
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="E52" s="11" t="n">
-        <v>536</v>
+        <v>537</v>
       </c>
     </row>
     <row r="53">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="E53" s="8" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="54">
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="E56" s="8" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="57">
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="E57" s="8" t="n">
-        <v>967</v>
+        <v>995</v>
       </c>
     </row>
     <row r="58">
@@ -1802,7 +1802,7 @@
         </is>
       </c>
       <c r="E58" s="8" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="59">
@@ -1850,7 +1850,7 @@
         </is>
       </c>
       <c r="E60" s="8" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="61">
@@ -1988,7 +1988,7 @@
         </is>
       </c>
       <c r="E66" s="8" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="67">
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="E67" s="8" t="n">
-        <v>1176</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="68">
@@ -2034,7 +2034,7 @@
         </is>
       </c>
       <c r="E68" s="8" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="69">
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="E69" s="8" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="70">
@@ -2157,7 +2157,7 @@
         </is>
       </c>
       <c r="E73" s="11" t="n">
-        <v>296</v>
+        <v>425</v>
       </c>
     </row>
     <row r="74">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="E79" s="11" t="n">
-        <v>207</v>
+        <v>240</v>
       </c>
     </row>
     <row r="80">
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="E85" s="11" t="n">
-        <v>81</v>
+        <v>110</v>
       </c>
     </row>
     <row r="86">
@@ -2728,7 +2728,7 @@
         </is>
       </c>
       <c r="E96" s="8" t="n">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="97">
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="E98" s="8" t="n">
-        <v>392</v>
+        <v>398</v>
       </c>
     </row>
     <row r="99">
@@ -2866,7 +2866,7 @@
         </is>
       </c>
       <c r="E102" s="8" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="103">
@@ -2935,7 +2935,7 @@
         </is>
       </c>
       <c r="E105" s="8" t="n">
-        <v>386</v>
+        <v>390</v>
       </c>
     </row>
     <row r="106">
@@ -2958,7 +2958,7 @@
         </is>
       </c>
       <c r="E106" s="8" t="n">
-        <v>26</v>
+        <v>43</v>
       </c>
     </row>
     <row r="107">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="E107" s="8" t="n">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="108">
@@ -3004,7 +3004,7 @@
         </is>
       </c>
       <c r="E108" s="8" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="109">
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="E115" s="11" t="n">
-        <v>124</v>
+        <v>140</v>
       </c>
     </row>
     <row r="116">
@@ -3196,7 +3196,7 @@
         </is>
       </c>
       <c r="E116" s="11" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="117">
@@ -3321,7 +3321,7 @@
         </is>
       </c>
       <c r="E121" s="11" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="122">
@@ -3344,7 +3344,7 @@
         </is>
       </c>
       <c r="E122" s="8" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="123">
@@ -3390,7 +3390,7 @@
         </is>
       </c>
       <c r="E124" s="8" t="n">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="125">
@@ -3413,7 +3413,7 @@
         </is>
       </c>
       <c r="E125" s="8" t="n">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="126">
@@ -3459,7 +3459,7 @@
         </is>
       </c>
       <c r="E127" s="8" t="n">
-        <v>1376</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="128">
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="E129" s="8" t="n">
-        <v>1906</v>
+        <v>1984</v>
       </c>
     </row>
     <row r="130">
@@ -3528,7 +3528,7 @@
         </is>
       </c>
       <c r="E130" s="8" t="n">
-        <v>1775</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="131">
@@ -3551,7 +3551,7 @@
         </is>
       </c>
       <c r="E131" s="8" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="132">
@@ -3574,7 +3574,7 @@
         </is>
       </c>
       <c r="E132" s="8" t="n">
-        <v>2618</v>
+        <v>2707</v>
       </c>
     </row>
     <row r="133">
@@ -3620,7 +3620,7 @@
         </is>
       </c>
       <c r="E134" s="8" t="n">
-        <v>1894</v>
+        <v>1940</v>
       </c>
     </row>
     <row r="135">
@@ -3643,7 +3643,7 @@
         </is>
       </c>
       <c r="E135" s="8" t="n">
-        <v>2268</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="136">
@@ -3741,7 +3741,7 @@
         </is>
       </c>
       <c r="E139" s="11" t="n">
-        <v>96</v>
+        <v>201</v>
       </c>
     </row>
     <row r="140">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="E141" s="8" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="142">
@@ -3810,7 +3810,7 @@
         </is>
       </c>
       <c r="E142" s="8" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="143">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="E145" s="8" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="146">
@@ -3971,7 +3971,7 @@
         </is>
       </c>
       <c r="E149" s="8" t="n">
-        <v>1107</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="150">
@@ -4040,7 +4040,7 @@
         </is>
       </c>
       <c r="E152" s="8" t="n">
-        <v>1113</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="153">
@@ -4063,7 +4063,7 @@
         </is>
       </c>
       <c r="E153" s="8" t="n">
-        <v>220</v>
+        <v>228</v>
       </c>
     </row>
     <row r="154">
@@ -4086,7 +4086,7 @@
         </is>
       </c>
       <c r="E154" s="8" t="n">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="155">
@@ -4109,7 +4109,7 @@
         </is>
       </c>
       <c r="E155" s="8" t="n">
-        <v>685</v>
+        <v>688</v>
       </c>
     </row>
     <row r="156">
@@ -4224,7 +4224,7 @@
         </is>
       </c>
       <c r="E160" s="8" t="n">
-        <v>2793</v>
+        <v>2880</v>
       </c>
     </row>
     <row r="161">
@@ -4247,7 +4247,7 @@
         </is>
       </c>
       <c r="E161" s="8" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="162">
@@ -4270,7 +4270,7 @@
         </is>
       </c>
       <c r="E162" s="8" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="163">
@@ -4293,7 +4293,7 @@
         </is>
       </c>
       <c r="E163" s="8" t="n">
-        <v>1124</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="164">
@@ -4385,7 +4385,7 @@
         </is>
       </c>
       <c r="E167" s="8" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="168">
@@ -4454,7 +4454,7 @@
         </is>
       </c>
       <c r="E170" s="8" t="n">
-        <v>1099</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="171">
@@ -4500,7 +4500,7 @@
         </is>
       </c>
       <c r="E172" s="8" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="173">
@@ -4523,7 +4523,7 @@
         </is>
       </c>
       <c r="E173" s="8" t="n">
-        <v>1232</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="174">
@@ -4569,7 +4569,7 @@
         </is>
       </c>
       <c r="E175" s="8" t="n">
-        <v>1216</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="176">
@@ -4615,7 +4615,7 @@
         </is>
       </c>
       <c r="E177" s="8" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="178">
@@ -4661,7 +4661,7 @@
         </is>
       </c>
       <c r="E179" s="8" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="180">
@@ -4684,7 +4684,7 @@
         </is>
       </c>
       <c r="E180" s="8" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="181">
@@ -4753,7 +4753,7 @@
         </is>
       </c>
       <c r="E183" s="8" t="n">
-        <v>1204</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="184">
@@ -4776,7 +4776,7 @@
         </is>
       </c>
       <c r="E184" s="8" t="n">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="185">
@@ -4845,7 +4845,7 @@
         </is>
       </c>
       <c r="E187" s="8" t="n">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="188">
@@ -4893,7 +4893,7 @@
         </is>
       </c>
       <c r="E189" s="8" t="n">
-        <v>290</v>
+        <v>304</v>
       </c>
     </row>
     <row r="190">
@@ -4939,7 +4939,7 @@
         </is>
       </c>
       <c r="E191" s="8" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="192">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="E192" s="8" t="n">
-        <v>808</v>
+        <v>810</v>
       </c>
     </row>
     <row r="193">
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="E194" s="8" t="n">
-        <v>594</v>
+        <v>595</v>
       </c>
     </row>
     <row r="195">
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="E195" s="8" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="196">
@@ -5054,7 +5054,7 @@
         </is>
       </c>
       <c r="E196" s="8" t="n">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="197">
@@ -5146,7 +5146,7 @@
         </is>
       </c>
       <c r="E200" s="8" t="n">
-        <v>1143</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="201">
@@ -5194,7 +5194,7 @@
         </is>
       </c>
       <c r="E202" s="11" t="n">
-        <v>352</v>
+        <v>360</v>
       </c>
     </row>
     <row r="203">
@@ -5359,7 +5359,7 @@
         </is>
       </c>
       <c r="E209" s="11" t="n">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="210">
@@ -5428,7 +5428,7 @@
         </is>
       </c>
       <c r="E212" s="8" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="213">
@@ -5474,7 +5474,7 @@
         </is>
       </c>
       <c r="E214" s="8" t="n">
-        <v>455</v>
+        <v>457</v>
       </c>
     </row>
     <row r="215">
@@ -5543,7 +5543,7 @@
         </is>
       </c>
       <c r="E217" s="8" t="n">
-        <v>1395</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="218">
@@ -5589,7 +5589,7 @@
         </is>
       </c>
       <c r="E219" s="8" t="n">
-        <v>2882</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="220">
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="E220" s="8" t="n">
-        <v>2788</v>
+        <v>2797</v>
       </c>
     </row>
     <row r="221">
@@ -5635,7 +5635,7 @@
         </is>
       </c>
       <c r="E221" s="8" t="n">
-        <v>2929</v>
+        <v>3017</v>
       </c>
     </row>
     <row r="222">
@@ -5658,7 +5658,7 @@
         </is>
       </c>
       <c r="E222" s="8" t="n">
-        <v>2750</v>
+        <v>2753</v>
       </c>
     </row>
     <row r="223">
@@ -5681,7 +5681,7 @@
         </is>
       </c>
       <c r="E223" s="8" t="n">
-        <v>459</v>
+        <v>470</v>
       </c>
     </row>
     <row r="224">
@@ -5727,7 +5727,7 @@
         </is>
       </c>
       <c r="E225" s="8" t="n">
-        <v>2766</v>
+        <v>2851</v>
       </c>
     </row>
     <row r="226">
@@ -5773,7 +5773,7 @@
         </is>
       </c>
       <c r="E227" s="8" t="n">
-        <v>1592</v>
+        <v>1594</v>
       </c>
     </row>
     <row r="228">
@@ -5796,7 +5796,7 @@
         </is>
       </c>
       <c r="E228" s="8" t="n">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="229">
@@ -5842,7 +5842,7 @@
         </is>
       </c>
       <c r="E230" s="8" t="n">
-        <v>3036</v>
+        <v>3119</v>
       </c>
     </row>
     <row r="231">
@@ -5888,7 +5888,7 @@
         </is>
       </c>
       <c r="E232" s="8" t="n">
-        <v>2728</v>
+        <v>2733</v>
       </c>
     </row>
     <row r="233">
@@ -5911,7 +5911,7 @@
         </is>
       </c>
       <c r="E233" s="8" t="n">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="234">
@@ -5957,7 +5957,7 @@
         </is>
       </c>
       <c r="E235" s="8" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="236">
@@ -6026,7 +6026,7 @@
         </is>
       </c>
       <c r="E238" s="8" t="n">
-        <v>549</v>
+        <v>634</v>
       </c>
     </row>
     <row r="239">
@@ -6049,7 +6049,7 @@
         </is>
       </c>
       <c r="E239" s="8" t="n">
-        <v>1224</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="240">
@@ -6072,7 +6072,7 @@
         </is>
       </c>
       <c r="E240" s="8" t="n">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="241">
@@ -6233,7 +6233,7 @@
         </is>
       </c>
       <c r="E247" s="8" t="n">
-        <v>1133</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="248">
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="E248" s="8" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
     </row>
     <row r="249">
@@ -6279,7 +6279,7 @@
         </is>
       </c>
       <c r="E249" s="8" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="250">
@@ -6304,7 +6304,7 @@
         </is>
       </c>
       <c r="E250" s="11" t="n">
-        <v>1458</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="251">
@@ -6327,7 +6327,7 @@
         </is>
       </c>
       <c r="E251" s="8" t="n">
-        <v>443</v>
+        <v>451</v>
       </c>
     </row>
     <row r="252">
@@ -6373,7 +6373,7 @@
         </is>
       </c>
       <c r="E253" s="8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="254">
@@ -6396,7 +6396,7 @@
         </is>
       </c>
       <c r="E254" s="8" t="n">
-        <v>788</v>
+        <v>791</v>
       </c>
     </row>
     <row r="255">
@@ -6488,7 +6488,7 @@
         </is>
       </c>
       <c r="E258" s="8" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="259">
@@ -6511,7 +6511,7 @@
         </is>
       </c>
       <c r="E259" s="8" t="n">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="260">
@@ -6674,7 +6674,7 @@
         </is>
       </c>
       <c r="E266" s="8" t="n">
-        <v>1247</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="267">

</xml_diff>